<commit_message>
Add themes and use-case presets
Seven palettes selected with a "Theme" row in the About sheet: navy,
forest, plum, slate, sunset, ocean, and a light one, paper. Everything
was already written against six colour names, so a theme is a palette
swap — except paper, which also has to undo the hero's white text and
shadows. An unrecognised name falls back to the default rather than
producing an unstyled page.

Six templates for different groups — society, school, club, team,
temple, alumni — each with its own sheets, columns and theme. A preset is
only a list of sheets and a theme, so adding one is a few lines.

Urgent-contact sheets are no longer required to be called Emergency:
"On Call", "Helpline" and "24x7" now get the same red sidebar, which a
team or a club is far more likely to use.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/directory-template.xlsx
+++ b/template/directory-template.xlsx
@@ -522,21 +522,21 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Hindi: Committee</v>
+        <v>Theme</v>
       </c>
       <c r="B11" t="str">
-        <v>समिति</v>
+        <v>navy</v>
       </c>
       <c r="C11" t="str">
-        <v>हिंदी में अनुभाग का नाम</v>
+        <v>navy, forest, plum, slate, sunset, ocean, paper</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Hindi: Emergency</v>
+        <v>Hindi: Committee</v>
       </c>
       <c r="B12" t="str">
-        <v>आपातकालीन संपर्क</v>
+        <v>समिति</v>
       </c>
       <c r="C12" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -544,10 +544,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Hindi: Services &amp; Help</v>
+        <v>Hindi: Emergency</v>
       </c>
       <c r="B13" t="str">
-        <v>सेवाएँ और सहायता</v>
+        <v>आपातकालीन संपर्क</v>
       </c>
       <c r="C13" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -555,10 +555,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Hindi: Residents</v>
+        <v>Hindi: Services &amp; Help</v>
       </c>
       <c r="B14" t="str">
-        <v>निवासी</v>
+        <v>सेवाएँ और सहायता</v>
       </c>
       <c r="C14" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Hindi: Documents</v>
+        <v>Hindi: Residents</v>
       </c>
       <c r="B15" t="str">
-        <v>दस्तावेज़</v>
+        <v>निवासी</v>
       </c>
       <c r="C15" t="str">
         <v>हिंदी में अनुभाग का नाम</v>
@@ -577,24 +577,24 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Note: Services &amp; Help</v>
+        <v>Hindi: Documents</v>
       </c>
       <c r="B16" t="str">
-        <v>These contacts are collected from fellow residents. The society has not verified or endorsed any of them. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
+        <v>दस्तावेज़</v>
       </c>
       <c r="C16" t="str">
-        <v>उस अनुभाग के नीचे दिखने वाली चेतावनी</v>
+        <v>हिंदी में अनुभाग का नाम</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Note HI: Services &amp; Help</v>
+        <v>Note: Services &amp; Help</v>
       </c>
       <c r="B17" t="str">
-        <v>ये संपर्क अन्य निवासियों द्वारा दिए गए हैं। सोसाइटी ने इनकी जाँच नहीं की है। काम शुरू कराने से पहले कृपया स्वयं पुष्टि करें और शुल्क तय कर लें — जोखिम आपका अपना होगा।</v>
+        <v>These contacts are collected from members. They have not been verified or endorsed. Please check credentials and agree charges before engaging anyone — you do so at your own risk.</v>
       </c>
       <c r="C17" t="str">
-        <v>वही चेतावनी हिंदी में</v>
+        <v>उस अनुभाग के नीचे दिखने वाली चेतावनी</v>
       </c>
     </row>
   </sheetData>

</xml_diff>